<commit_message>
update readings for tues
</commit_message>
<xml_diff>
--- a/ids720_specific/class_schedule_720_xlsx.xlsx
+++ b/ids720_specific/class_schedule_720_xlsx.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nce8/github/practicaldatascience_book/ids720_specific/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0CAC6F-E55F-2F4D-BE5F-6591397BBE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A530E782-5B17-5F4E-9C41-E7C14F4960CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -211,14 +211,6 @@
     <t>Tues, Oct 6</t>
   </si>
   <si>
-    <t>- `Plotting in Python through seaborn and Grammer of Graphics &lt;../notebooks/class_5/week_1/2.3.1_plotting_with_seaborn.html&gt;`_
-- `seaborn recipes &lt;../notebooks/class_5/week_1/2.3.2_seaborn_recipes.html&gt;`_
-- `Customizing matplotlib &lt;../notebooks/class_5/week_1/2.1.2_customizing_plot_styles.html&gt;`_
-- `Making Pretty Plots 1 &lt;../notebooks/class_5/week_1/2.2.1_making_plots_pretty_1.html&gt;`_
-- `Making Pretty Plots 2 &lt;../notebooks/class_5/week_1/2.2.2_making_plots_pretty_2.html&gt;`_
-- `Pandas Plotting &lt;../notebooks/class_5/week_1/1.6.1_plotting_with_pandas.html&gt;`_</t>
-  </si>
-  <si>
     <t>- `Link &lt;../exercises/exercise_plotting_part2.html&gt;`_</t>
   </si>
   <si>
@@ -418,6 +410,15 @@
   <si>
     <t>- `Ex 1 &lt;../exercises/exercise_debugger720.html&gt;`_
 - `Ex 2 &lt;../exercises/exercise_variables_v_objects.html&gt;`_</t>
+  </si>
+  <si>
+    <t>- `Principles of AI &lt;https://dukemids.com/data_science_skills/principles_of_effective_ai_use.html&gt;`_
+- `Plotting in Python through seaborn and Grammer of Graphics &lt;../notebooks/class_5/week_1/2.3.1_plotting_with_seaborn.html&gt;`_
+- `seaborn recipes &lt;../notebooks/class_5/week_1/2.3.2_seaborn_recipes.html&gt;`_
+- `Customizing matplotlib &lt;../notebooks/class_5/week_1/2.1.2_customizing_plot_styles.html&gt;`_
+- `Making Pretty Plots 1 &lt;../notebooks/class_5/week_1/2.2.1_making_plots_pretty_1.html&gt;`_
+- `Making Pretty Plots 2 &lt;../notebooks/class_5/week_1/2.2.2_making_plots_pretty_2.html&gt;`_
+- `Pandas Plotting &lt;../notebooks/class_5/week_1/1.6.1_plotting_with_pandas.html&gt;`_</t>
   </si>
 </sst>
 </file>
@@ -854,7 +855,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D2" s="8"/>
     </row>
@@ -880,7 +881,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>12</v>
@@ -897,7 +898,7 @@
         <v>15</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="136" customHeight="1" x14ac:dyDescent="0.2">
@@ -911,7 +912,7 @@
         <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="85" customHeight="1" x14ac:dyDescent="0.2">
@@ -925,7 +926,7 @@
         <v>21</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="272" customHeight="1" x14ac:dyDescent="0.2">
@@ -1012,7 +1013,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="142" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13" t="s">
         <v>46</v>
       </c>
@@ -1020,183 +1021,183 @@
         <v>43</v>
       </c>
       <c r="C14" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="102" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="D15" s="9" t="s">
         <v>51</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
         <v>53</v>
-      </c>
-      <c r="B16" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" t="s">
         <v>55</v>
-      </c>
-      <c r="B17" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="D18" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="D19" s="15" t="s">
         <v>63</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="43" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="106" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="C21" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>70</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="140" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="C22" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="8" t="s">
         <v>74</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="8" t="s">
         <v>77</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>78</v>
       </c>
       <c r="D23" s="7"/>
     </row>
     <row r="24" spans="1:4" ht="134" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="103" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="C25" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="C26" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="D26" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" t="s">
         <v>91</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>94</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>